<commit_message>
Add dataset-origin plots and 2025 results summary
</commit_message>
<xml_diff>
--- a/workbooks/2025/AD_2025_analysis.xlsx
+++ b/workbooks/2025/AD_2025_analysis.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>916</v>
+        <v>913</v>
       </c>
     </row>
     <row r="4">
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>916</v>
+        <v>913</v>
       </c>
     </row>
     <row r="5">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>813</v>
+        <v>810</v>
       </c>
     </row>
     <row r="8">
@@ -499,7 +499,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>88.8%</t>
+          <t>88.7%</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>812</v>
+        <v>809</v>
       </c>
     </row>
     <row r="12">
@@ -555,7 +555,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>3.0%</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>813</v>
+        <v>810</v>
       </c>
     </row>
     <row r="16">
@@ -577,7 +577,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>88.8%</t>
+          <t>88.7%</t>
         </is>
       </c>
     </row>
@@ -596,126 +596,116 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other</t>
+          <t xml:space="preserve">  GitHub</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>827</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GitHub</t>
+          <t xml:space="preserve">  OSF</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  OSF</t>
+          <t xml:space="preserve">  Zenodo</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Zenodo</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>2</v>
-      </c>
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>--- SEX-SPECIFIC ANALYSIS ---</t>
+        </is>
+      </c>
       <c r="B23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>--- SEX-SPECIFIC ANALYSIS ---</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>Papers with sex-specific keywords</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>233</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Papers with sex-specific keywords</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>233</v>
+          <t>% papers with sex analysis</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>25.5%</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>% papers with sex analysis</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>25.4%</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>--- COUNTRY ---</t>
+        </is>
+      </c>
       <c r="B27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>--- COUNTRY ---</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>Papers with country identified</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>905</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Papers with country identified</t>
+          <t>Chi-square (country × sharing)</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>908</v>
+        <v>9.592000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Chi-square (country × sharing)</t>
+          <t>p-value</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9.605</v>
+        <v>0.3845</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>p-value</t>
+          <t>Cramér's V</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.3834</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Cramér's V</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
         <v>0.105</v>
       </c>
     </row>
@@ -762,10 +752,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="C2" t="n">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="D2" t="n">
         <v>88.5</v>

</xml_diff>